<commit_message>
Run4 with leadlag calculations
</commit_message>
<xml_diff>
--- a/parameters_CCM.xlsx
+++ b/parameters_CCM.xlsx
@@ -1,21 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonro\OneDrive\Desktop\Algal_blooms\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b94c59a01e372ca2/Desktop/Algal_blooms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A267BACA-5322-4D14-AD98-2B8644D6D7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="664" documentId="8_{A267BACA-5322-4D14-AD98-2B8644D6D7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A58853B-7C77-40FD-80C3-A02D1D1C5798}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="2" xr2:uid="{96C955FB-9A51-4D0B-AF49-129559A448B6}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{96C955FB-9A51-4D0B-AF49-129559A448B6}"/>
   </bookViews>
   <sheets>
     <sheet name="Run1" sheetId="1" r:id="rId1"/>
     <sheet name="Run2" sheetId="2" r:id="rId2"/>
     <sheet name="Run3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sat" sheetId="4" r:id="rId4"/>
+    <sheet name="Run4" sheetId="5" r:id="rId5"/>
+    <sheet name="Surrogate_results" sheetId="6" r:id="rId6"/>
+    <sheet name="leadlag_results" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="72">
   <si>
     <t>Variable</t>
   </si>
@@ -170,6 +174,90 @@
   </si>
   <si>
     <t>acminstage</t>
+  </si>
+  <si>
+    <t>Area</t>
+  </si>
+  <si>
+    <t>easting</t>
+  </si>
+  <si>
+    <t>northing</t>
+  </si>
+  <si>
+    <t>Yish?</t>
+  </si>
+  <si>
+    <t>wind speed</t>
+  </si>
+  <si>
+    <t>wind dir</t>
+  </si>
+  <si>
+    <t>mctn</t>
+  </si>
+  <si>
+    <t>mctp</t>
+  </si>
+  <si>
+    <t>mcnh4</t>
+  </si>
+  <si>
+    <t>mcdoc</t>
+  </si>
+  <si>
+    <t>mcsal</t>
+  </si>
+  <si>
+    <t>mflow</t>
+  </si>
+  <si>
+    <t>mmaxstage</t>
+  </si>
+  <si>
+    <t>rsal</t>
+  </si>
+  <si>
+    <t>rchl</t>
+  </si>
+  <si>
+    <t>marshmeanrain</t>
+  </si>
+  <si>
+    <t>Stationarity (nce)</t>
+  </si>
+  <si>
+    <t>Effect</t>
+  </si>
+  <si>
+    <t>Cause</t>
+  </si>
+  <si>
+    <t>p-value</t>
+  </si>
+  <si>
+    <t>area</t>
+  </si>
+  <si>
+    <t>WD</t>
+  </si>
+  <si>
+    <t>Highest rho</t>
+  </si>
+  <si>
+    <t>leadlag</t>
+  </si>
+  <si>
+    <t>use</t>
+  </si>
+  <si>
+    <t>dir</t>
+  </si>
+  <si>
+    <t>speed</t>
+  </si>
+  <si>
+    <t>Surrogate_sig</t>
   </si>
 </sst>
 </file>
@@ -229,6 +317,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1520,4 +1612,2656 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59E1CC5D-6164-4A94-8A65-479138E1B71D}">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="2" max="2" width="21.453125" customWidth="1"/>
+    <col min="3" max="3" width="21.81640625" customWidth="1"/>
+    <col min="4" max="4" width="23.90625" customWidth="1"/>
+    <col min="5" max="5" width="13.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="1">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="1">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1">
+        <v>4</v>
+      </c>
+      <c r="D4" s="1">
+        <v>3</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="1">
+        <v>2</v>
+      </c>
+      <c r="C5" s="1">
+        <v>3</v>
+      </c>
+      <c r="D5" s="1">
+        <v>2</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" s="1">
+        <v>4</v>
+      </c>
+      <c r="C6" s="1">
+        <v>4</v>
+      </c>
+      <c r="D6" s="1">
+        <v>3</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0219A31A-9904-40E1-98EE-E1AAB97C02AB}">
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="16.08984375" customWidth="1"/>
+    <col min="2" max="2" width="17.36328125" customWidth="1"/>
+    <col min="3" max="3" width="16.36328125" customWidth="1"/>
+    <col min="4" max="4" width="24.7265625" customWidth="1"/>
+    <col min="5" max="5" width="15.54296875" customWidth="1"/>
+    <col min="6" max="6" width="12.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2</v>
+      </c>
+      <c r="D4" s="1">
+        <v>4</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" s="1">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1">
+        <v>3</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="1">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1">
+        <v>4</v>
+      </c>
+      <c r="D7" s="1">
+        <v>3</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="1">
+        <v>2</v>
+      </c>
+      <c r="C8" s="1">
+        <v>4</v>
+      </c>
+      <c r="D8" s="1">
+        <v>3</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="1">
+        <v>2</v>
+      </c>
+      <c r="C9" s="1">
+        <v>3</v>
+      </c>
+      <c r="D9" s="1">
+        <v>4</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" s="1">
+        <v>5</v>
+      </c>
+      <c r="C10" s="1">
+        <v>4</v>
+      </c>
+      <c r="D10" s="1">
+        <v>4</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="1">
+        <v>2</v>
+      </c>
+      <c r="C11" s="1">
+        <v>3</v>
+      </c>
+      <c r="D11" s="1">
+        <v>3</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="1">
+        <v>4</v>
+      </c>
+      <c r="C12" s="1">
+        <v>3</v>
+      </c>
+      <c r="D12" s="1">
+        <v>3</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" s="1">
+        <v>2</v>
+      </c>
+      <c r="C13" s="1">
+        <v>3</v>
+      </c>
+      <c r="D13" s="1">
+        <v>3</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="1">
+        <v>2</v>
+      </c>
+      <c r="C14" s="1">
+        <v>3</v>
+      </c>
+      <c r="D14" s="1">
+        <v>2</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" s="1">
+        <v>3</v>
+      </c>
+      <c r="C15" s="1">
+        <v>3</v>
+      </c>
+      <c r="D15" s="1">
+        <v>4</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="1">
+        <v>5</v>
+      </c>
+      <c r="C16" s="1">
+        <v>7</v>
+      </c>
+      <c r="D16" s="1">
+        <v>4</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="1">
+        <v>5</v>
+      </c>
+      <c r="C17" s="1">
+        <v>10</v>
+      </c>
+      <c r="D17" s="1">
+        <v>5</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="1">
+        <v>5</v>
+      </c>
+      <c r="C18" s="1">
+        <v>4</v>
+      </c>
+      <c r="D18" s="1">
+        <v>4</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19">
+        <v>4</v>
+      </c>
+      <c r="C19">
+        <v>3</v>
+      </c>
+      <c r="D19">
+        <v>4</v>
+      </c>
+      <c r="E19" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" s="1">
+        <v>3</v>
+      </c>
+      <c r="C20" s="1">
+        <v>4</v>
+      </c>
+      <c r="D20" s="1">
+        <v>4</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21">
+        <v>4</v>
+      </c>
+      <c r="C21">
+        <v>7</v>
+      </c>
+      <c r="D21">
+        <v>4</v>
+      </c>
+      <c r="E21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22">
+        <v>4</v>
+      </c>
+      <c r="E22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>34</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>2</v>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
+      <c r="E23" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B24" s="1">
+        <v>4</v>
+      </c>
+      <c r="C24" s="1">
+        <v>3</v>
+      </c>
+      <c r="D24" s="1">
+        <v>3</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>3</v>
+      </c>
+      <c r="C25">
+        <v>4</v>
+      </c>
+      <c r="D25">
+        <v>3</v>
+      </c>
+      <c r="E25" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="1">
+        <v>3</v>
+      </c>
+      <c r="C26" s="1">
+        <v>2</v>
+      </c>
+      <c r="D26" s="1">
+        <v>3</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1">
+        <v>1</v>
+      </c>
+      <c r="C27" s="1">
+        <v>2</v>
+      </c>
+      <c r="D27" s="1">
+        <v>3</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28" s="1">
+        <v>2</v>
+      </c>
+      <c r="C28" s="1">
+        <v>3</v>
+      </c>
+      <c r="D28" s="1">
+        <v>3</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" s="1">
+        <v>3</v>
+      </c>
+      <c r="C29" s="1">
+        <v>3</v>
+      </c>
+      <c r="D29" s="1">
+        <v>2</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="1">
+        <v>4</v>
+      </c>
+      <c r="C30" s="1">
+        <v>3</v>
+      </c>
+      <c r="D30" s="1">
+        <v>3</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F30" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D34DCF9A-2763-4D42-B469-B0C248749245}">
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="18.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1">
+        <v>7.9799999999999992E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1.99E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="1">
+        <v>3.7900000000000003E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="1">
+        <v>6.9800000000000001E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="1">
+        <v>1.99E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7">
+        <v>0.17799999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" s="1">
+        <v>5.3999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9">
+        <v>0.30499999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="1">
+        <v>9.8699999999999996E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11">
+        <v>0.104</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="1">
+        <v>7.5800000000000006E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="1">
+        <v>4.99E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="1">
+        <v>4.7899999999999998E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15">
+        <v>0.13900000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" s="1">
+        <v>1.99E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="1">
+        <v>2E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B18" t="s">
+        <v>65</v>
+      </c>
+      <c r="C18">
+        <v>0.22500000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4796A85C-8317-4493-888D-443234A7E4BB}">
+  <dimension ref="A1:F104"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="2" width="16.81640625" customWidth="1"/>
+    <col min="3" max="3" width="19.6328125" customWidth="1"/>
+    <col min="4" max="4" width="19.36328125" customWidth="1"/>
+    <col min="5" max="5" width="17.453125" customWidth="1"/>
+    <col min="6" max="6" width="15.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.30499999999999999</v>
+      </c>
+      <c r="D2" s="1">
+        <v>-4</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3">
+        <v>0.14599999999999999</v>
+      </c>
+      <c r="D3">
+        <v>6</v>
+      </c>
+      <c r="E3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4">
+        <v>0.128</v>
+      </c>
+      <c r="D4">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.35299999999999998</v>
+      </c>
+      <c r="D5" s="1">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.36799999999999999</v>
+      </c>
+      <c r="D6" s="1">
+        <v>7</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.42599999999999999</v>
+      </c>
+      <c r="D7" s="1">
+        <v>9</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8">
+        <v>0.32</v>
+      </c>
+      <c r="D8">
+        <v>-12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="1">
+        <v>0.45900000000000002</v>
+      </c>
+      <c r="D9" s="1">
+        <v>10</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10">
+        <v>0.253</v>
+      </c>
+      <c r="D10">
+        <v>-4</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="1">
+        <v>0.39400000000000002</v>
+      </c>
+      <c r="D11" s="1">
+        <v>7</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12">
+        <v>0.20300000000000001</v>
+      </c>
+      <c r="D12">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13">
+        <v>0.22600000000000001</v>
+      </c>
+      <c r="D13">
+        <v>-8</v>
+      </c>
+      <c r="E13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="D14" s="1">
+        <v>-7</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15">
+        <v>0.13600000000000001</v>
+      </c>
+      <c r="D15">
+        <v>-2</v>
+      </c>
+      <c r="E15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="1">
+        <v>0.29099999999999998</v>
+      </c>
+      <c r="D16" s="1">
+        <v>6</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0.375</v>
+      </c>
+      <c r="D17" s="1">
+        <v>-2</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18">
+        <v>0.20100000000000001</v>
+      </c>
+      <c r="D18">
+        <v>-3</v>
+      </c>
+      <c r="E18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0.46200000000000002</v>
+      </c>
+      <c r="D19" s="1">
+        <v>2</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C20" s="1">
+        <v>0.311</v>
+      </c>
+      <c r="D20" s="1">
+        <v>0</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="D21">
+        <v>10</v>
+      </c>
+      <c r="E21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" s="1">
+        <v>0.47299999999999998</v>
+      </c>
+      <c r="D22" s="1">
+        <v>-4</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="1">
+        <v>0.48099999999999998</v>
+      </c>
+      <c r="D23" s="1">
+        <v>6</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24">
+        <v>0.255</v>
+      </c>
+      <c r="D24">
+        <v>7</v>
+      </c>
+      <c r="E24" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" s="1">
+        <v>0.61</v>
+      </c>
+      <c r="D25" s="1">
+        <v>0</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" s="1">
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D26" s="1">
+        <v>0</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C27" s="1">
+        <v>0.51800000000000002</v>
+      </c>
+      <c r="D27" s="1">
+        <v>0</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C28" s="1">
+        <v>0.311</v>
+      </c>
+      <c r="D28" s="1">
+        <v>-3</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>4</v>
+      </c>
+      <c r="B29" t="s">
+        <v>11</v>
+      </c>
+      <c r="C29">
+        <v>0.111</v>
+      </c>
+      <c r="D29">
+        <v>-12</v>
+      </c>
+      <c r="E29" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" t="s">
+        <v>7</v>
+      </c>
+      <c r="C30">
+        <v>0.38</v>
+      </c>
+      <c r="D30">
+        <v>-12</v>
+      </c>
+      <c r="E30" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31">
+        <v>0.28499999999999998</v>
+      </c>
+      <c r="D31">
+        <v>-12</v>
+      </c>
+      <c r="E31" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" s="1">
+        <v>0.33300000000000002</v>
+      </c>
+      <c r="D32" s="1">
+        <v>6</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" t="s">
+        <v>31</v>
+      </c>
+      <c r="C33">
+        <v>0.16800000000000001</v>
+      </c>
+      <c r="D33">
+        <v>5</v>
+      </c>
+      <c r="E33" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" t="s">
+        <v>69</v>
+      </c>
+      <c r="C34">
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="D34">
+        <v>2</v>
+      </c>
+      <c r="E34" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C35" s="1">
+        <v>0.223</v>
+      </c>
+      <c r="D35" s="1">
+        <v>-4</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C36" s="1">
+        <v>0.47</v>
+      </c>
+      <c r="D36" s="1">
+        <v>-4</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="D37" s="1">
+        <v>7</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>4</v>
+      </c>
+      <c r="B38" t="s">
+        <v>28</v>
+      </c>
+      <c r="C38">
+        <v>0.192</v>
+      </c>
+      <c r="D38">
+        <v>5</v>
+      </c>
+      <c r="E38" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>4</v>
+      </c>
+      <c r="B39" t="s">
+        <v>27</v>
+      </c>
+      <c r="C39">
+        <v>-0.154</v>
+      </c>
+      <c r="D39">
+        <v>9</v>
+      </c>
+      <c r="E39" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C40" s="1">
+        <v>0.496</v>
+      </c>
+      <c r="D40" s="1">
+        <v>-8</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C41" s="1">
+        <v>0.45600000000000002</v>
+      </c>
+      <c r="D41" s="1">
+        <v>8</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C42" s="1">
+        <v>0.73</v>
+      </c>
+      <c r="D42" s="1">
+        <v>-10</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>4</v>
+      </c>
+      <c r="B43" t="s">
+        <v>59</v>
+      </c>
+      <c r="C43">
+        <v>-0.13600000000000001</v>
+      </c>
+      <c r="D43">
+        <v>9</v>
+      </c>
+      <c r="E43" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>4</v>
+      </c>
+      <c r="B44" t="s">
+        <v>53</v>
+      </c>
+      <c r="C44">
+        <v>0.39800000000000002</v>
+      </c>
+      <c r="D44">
+        <v>9</v>
+      </c>
+      <c r="E44" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C45" s="1">
+        <v>0.503</v>
+      </c>
+      <c r="D45" s="1">
+        <v>-12</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>4</v>
+      </c>
+      <c r="B46" t="s">
+        <v>55</v>
+      </c>
+      <c r="C46">
+        <v>0.313</v>
+      </c>
+      <c r="D46">
+        <v>7</v>
+      </c>
+      <c r="E46" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>4</v>
+      </c>
+      <c r="B47" t="s">
+        <v>56</v>
+      </c>
+      <c r="C47">
+        <v>0.24099999999999999</v>
+      </c>
+      <c r="D47">
+        <v>5</v>
+      </c>
+      <c r="E47" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C48" s="1">
+        <v>0.29199999999999998</v>
+      </c>
+      <c r="D48" s="1">
+        <v>1</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>4</v>
+      </c>
+      <c r="B49" t="s">
+        <v>58</v>
+      </c>
+      <c r="C49">
+        <v>-4.0000000000000001E-3</v>
+      </c>
+      <c r="D49">
+        <v>-1</v>
+      </c>
+      <c r="E49" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>4</v>
+      </c>
+      <c r="B50" t="s">
+        <v>24</v>
+      </c>
+      <c r="C50">
+        <v>0.25900000000000001</v>
+      </c>
+      <c r="D50">
+        <v>-5</v>
+      </c>
+      <c r="E50" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C51" s="1">
+        <v>0.63600000000000001</v>
+      </c>
+      <c r="D51" s="1">
+        <v>7</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>4</v>
+      </c>
+      <c r="B52" t="s">
+        <v>26</v>
+      </c>
+      <c r="C52">
+        <v>5.8999999999999997E-2</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>4</v>
+      </c>
+      <c r="B53" t="s">
+        <v>33</v>
+      </c>
+      <c r="C53">
+        <v>0.32900000000000001</v>
+      </c>
+      <c r="D53">
+        <v>-4</v>
+      </c>
+      <c r="E53" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>4</v>
+      </c>
+      <c r="B54" t="s">
+        <v>34</v>
+      </c>
+      <c r="C54">
+        <v>6.7000000000000004E-2</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="E54" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>4</v>
+      </c>
+      <c r="B55" t="s">
+        <v>70</v>
+      </c>
+      <c r="C55">
+        <v>-3.3000000000000002E-2</v>
+      </c>
+      <c r="D55">
+        <v>4</v>
+      </c>
+      <c r="E55" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C56" s="1">
+        <v>0.36299999999999999</v>
+      </c>
+      <c r="D56" s="1">
+        <v>-7</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C57" s="1">
+        <v>0.38500000000000001</v>
+      </c>
+      <c r="D57" s="1">
+        <v>6</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>46</v>
+      </c>
+      <c r="B58" t="s">
+        <v>8</v>
+      </c>
+      <c r="C58">
+        <v>5.8000000000000003E-2</v>
+      </c>
+      <c r="D58">
+        <v>6</v>
+      </c>
+      <c r="E58" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>46</v>
+      </c>
+      <c r="B59" t="s">
+        <v>12</v>
+      </c>
+      <c r="C59">
+        <v>8.6999999999999994E-2</v>
+      </c>
+      <c r="D59">
+        <v>-2</v>
+      </c>
+      <c r="E59" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>46</v>
+      </c>
+      <c r="B60" t="s">
+        <v>31</v>
+      </c>
+      <c r="C60">
+        <v>0.35</v>
+      </c>
+      <c r="D60">
+        <v>9</v>
+      </c>
+      <c r="E60" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>46</v>
+      </c>
+      <c r="B61" t="s">
+        <v>64</v>
+      </c>
+      <c r="C61">
+        <v>0.17199999999999999</v>
+      </c>
+      <c r="D61">
+        <v>-2</v>
+      </c>
+      <c r="E61" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>46</v>
+      </c>
+      <c r="B62" t="s">
+        <v>69</v>
+      </c>
+      <c r="C62">
+        <v>0.111</v>
+      </c>
+      <c r="D62">
+        <v>12</v>
+      </c>
+      <c r="E62" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>46</v>
+      </c>
+      <c r="B63" t="s">
+        <v>28</v>
+      </c>
+      <c r="C63">
+        <v>0.191</v>
+      </c>
+      <c r="D63">
+        <v>-2</v>
+      </c>
+      <c r="E63" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A64" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C64" s="1">
+        <v>0.47699999999999998</v>
+      </c>
+      <c r="D64" s="1">
+        <v>6</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A65" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C65" s="1">
+        <v>0.318</v>
+      </c>
+      <c r="D65" s="1">
+        <v>9</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A66" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C66" s="1">
+        <v>0.51800000000000002</v>
+      </c>
+      <c r="D66" s="1">
+        <v>7</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>46</v>
+      </c>
+      <c r="B67" t="s">
+        <v>59</v>
+      </c>
+      <c r="C67">
+        <v>0.121</v>
+      </c>
+      <c r="D67">
+        <v>-12</v>
+      </c>
+      <c r="E67" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>46</v>
+      </c>
+      <c r="B68" t="s">
+        <v>53</v>
+      </c>
+      <c r="C68">
+        <v>0.36299999999999999</v>
+      </c>
+      <c r="D68">
+        <v>8</v>
+      </c>
+      <c r="E68" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>46</v>
+      </c>
+      <c r="B69" t="s">
+        <v>50</v>
+      </c>
+      <c r="C69">
+        <v>0.221</v>
+      </c>
+      <c r="D69">
+        <v>1</v>
+      </c>
+      <c r="E69" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>46</v>
+      </c>
+      <c r="B70" t="s">
+        <v>55</v>
+      </c>
+      <c r="C70">
+        <v>0.14399999999999999</v>
+      </c>
+      <c r="D70">
+        <v>12</v>
+      </c>
+      <c r="E70" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>46</v>
+      </c>
+      <c r="B71" t="s">
+        <v>56</v>
+      </c>
+      <c r="C71">
+        <v>0.189</v>
+      </c>
+      <c r="D71">
+        <v>-2</v>
+      </c>
+      <c r="E71" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>46</v>
+      </c>
+      <c r="B72" t="s">
+        <v>58</v>
+      </c>
+      <c r="C72">
+        <v>0.04</v>
+      </c>
+      <c r="D72">
+        <v>4</v>
+      </c>
+      <c r="E72" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A73" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C73" s="1">
+        <v>0.38400000000000001</v>
+      </c>
+      <c r="D73" s="1">
+        <v>-3</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>46</v>
+      </c>
+      <c r="B74" t="s">
+        <v>26</v>
+      </c>
+      <c r="C74">
+        <v>0.23</v>
+      </c>
+      <c r="D74">
+        <v>1</v>
+      </c>
+      <c r="E74" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>46</v>
+      </c>
+      <c r="B75" t="s">
+        <v>33</v>
+      </c>
+      <c r="C75">
+        <v>0.255</v>
+      </c>
+      <c r="D75">
+        <v>4</v>
+      </c>
+      <c r="E75" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>46</v>
+      </c>
+      <c r="B76" t="s">
+        <v>34</v>
+      </c>
+      <c r="C76">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="D76">
+        <v>4</v>
+      </c>
+      <c r="E76" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>46</v>
+      </c>
+      <c r="B77" t="s">
+        <v>70</v>
+      </c>
+      <c r="C77">
+        <v>0.26600000000000001</v>
+      </c>
+      <c r="D77">
+        <v>-11</v>
+      </c>
+      <c r="E77" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>58</v>
+      </c>
+      <c r="B78" t="s">
+        <v>11</v>
+      </c>
+      <c r="C78">
+        <v>8.1000000000000003E-2</v>
+      </c>
+      <c r="D78">
+        <v>0</v>
+      </c>
+      <c r="E78" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>58</v>
+      </c>
+      <c r="B79" t="s">
+        <v>7</v>
+      </c>
+      <c r="C79">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="D79">
+        <v>-10</v>
+      </c>
+      <c r="E79" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>58</v>
+      </c>
+      <c r="B80" t="s">
+        <v>8</v>
+      </c>
+      <c r="C80">
+        <v>2.9000000000000001E-2</v>
+      </c>
+      <c r="D80">
+        <v>-3</v>
+      </c>
+      <c r="E80" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>58</v>
+      </c>
+      <c r="B81" t="s">
+        <v>12</v>
+      </c>
+      <c r="C81">
+        <v>0.23300000000000001</v>
+      </c>
+      <c r="D81">
+        <v>2</v>
+      </c>
+      <c r="E81" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>58</v>
+      </c>
+      <c r="B82" t="s">
+        <v>31</v>
+      </c>
+      <c r="C82">
+        <v>0.20200000000000001</v>
+      </c>
+      <c r="D82">
+        <v>1</v>
+      </c>
+      <c r="E82" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>58</v>
+      </c>
+      <c r="B83" t="s">
+        <v>69</v>
+      </c>
+      <c r="C83">
+        <v>0.36499999999999999</v>
+      </c>
+      <c r="D83">
+        <v>11</v>
+      </c>
+      <c r="E83" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A84" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C84" s="1">
+        <v>0.61799999999999999</v>
+      </c>
+      <c r="D84" s="1">
+        <v>-6</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>58</v>
+      </c>
+      <c r="B85" t="s">
+        <v>22</v>
+      </c>
+      <c r="C85">
+        <v>0.20699999999999999</v>
+      </c>
+      <c r="D85">
+        <v>5</v>
+      </c>
+      <c r="E85" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A86" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C86" s="1">
+        <v>0.35399999999999998</v>
+      </c>
+      <c r="D86" s="1">
+        <v>1</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>58</v>
+      </c>
+      <c r="B87" t="s">
+        <v>28</v>
+      </c>
+      <c r="C87">
+        <v>0.193</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>58</v>
+      </c>
+      <c r="B88" t="s">
+        <v>27</v>
+      </c>
+      <c r="C88">
+        <v>0.02</v>
+      </c>
+      <c r="D88">
+        <v>8</v>
+      </c>
+      <c r="E88" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A89" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C89" s="1">
+        <v>0.40699999999999997</v>
+      </c>
+      <c r="D89" s="1">
+        <v>-11</v>
+      </c>
+      <c r="E89" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A90" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C90" s="1">
+        <v>0.27400000000000002</v>
+      </c>
+      <c r="D90" s="1">
+        <v>-9</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A91" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C91" s="1">
+        <v>0.35</v>
+      </c>
+      <c r="D91" s="1">
+        <v>-10</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>58</v>
+      </c>
+      <c r="B92" t="s">
+        <v>59</v>
+      </c>
+      <c r="C92">
+        <v>0.13100000000000001</v>
+      </c>
+      <c r="D92">
+        <v>5</v>
+      </c>
+      <c r="E92" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>58</v>
+      </c>
+      <c r="B93" t="s">
+        <v>53</v>
+      </c>
+      <c r="C93">
+        <v>0.33800000000000002</v>
+      </c>
+      <c r="D93">
+        <v>-11</v>
+      </c>
+      <c r="E93" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>58</v>
+      </c>
+      <c r="B94" t="s">
+        <v>50</v>
+      </c>
+      <c r="C94">
+        <v>0.16300000000000001</v>
+      </c>
+      <c r="D94">
+        <v>-11</v>
+      </c>
+      <c r="E94" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>58</v>
+      </c>
+      <c r="B95" t="s">
+        <v>55</v>
+      </c>
+      <c r="C95">
+        <v>0.17899999999999999</v>
+      </c>
+      <c r="D95">
+        <v>1</v>
+      </c>
+      <c r="E95" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>58</v>
+      </c>
+      <c r="B96" t="s">
+        <v>56</v>
+      </c>
+      <c r="C96">
+        <v>0.23499999999999999</v>
+      </c>
+      <c r="D96">
+        <v>1</v>
+      </c>
+      <c r="E96" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>58</v>
+      </c>
+      <c r="B97" t="s">
+        <v>46</v>
+      </c>
+      <c r="C97">
+        <v>0.21299999999999999</v>
+      </c>
+      <c r="D97">
+        <v>11</v>
+      </c>
+      <c r="E97" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A98" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C98" s="1">
+        <v>0.34100000000000003</v>
+      </c>
+      <c r="D98" s="1">
+        <v>-11</v>
+      </c>
+      <c r="E98" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>58</v>
+      </c>
+      <c r="B99" t="s">
+        <v>24</v>
+      </c>
+      <c r="C99">
+        <v>0.20899999999999999</v>
+      </c>
+      <c r="D99">
+        <v>9</v>
+      </c>
+      <c r="E99" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>58</v>
+      </c>
+      <c r="B100" t="s">
+        <v>57</v>
+      </c>
+      <c r="C100">
+        <v>0.156</v>
+      </c>
+      <c r="D100">
+        <v>8</v>
+      </c>
+      <c r="E100" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A101" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C101" s="1">
+        <v>0.70399999999999996</v>
+      </c>
+      <c r="D101" s="1">
+        <v>0</v>
+      </c>
+      <c r="E101" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A102" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C102" s="1">
+        <v>0.48899999999999999</v>
+      </c>
+      <c r="D102" s="1">
+        <v>0</v>
+      </c>
+      <c r="E102" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A103" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C103" s="1">
+        <v>0.73699999999999999</v>
+      </c>
+      <c r="D103" s="1">
+        <v>0</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>58</v>
+      </c>
+      <c r="B104" t="s">
+        <v>70</v>
+      </c>
+      <c r="C104">
+        <v>5.8000000000000003E-2</v>
+      </c>
+      <c r="D104">
+        <v>4</v>
+      </c>
+      <c r="E104" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Figures of lagged effects
</commit_message>
<xml_diff>
--- a/parameters_CCM.xlsx
+++ b/parameters_CCM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b94c59a01e372ca2/Desktop/Algal_blooms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="728" documentId="8_{A267BACA-5322-4D14-AD98-2B8644D6D7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37D37E42-9DA2-45CD-89A9-C21BDBCB0E65}"/>
+  <xr:revisionPtr revIDLastSave="781" documentId="8_{A267BACA-5322-4D14-AD98-2B8644D6D7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C36811B-19E7-478D-8061-DECCF14C2683}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="6" xr2:uid="{96C955FB-9A51-4D0B-AF49-129559A448B6}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" activeTab="6" xr2:uid="{96C955FB-9A51-4D0B-AF49-129559A448B6}"/>
   </bookViews>
   <sheets>
     <sheet name="Run1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="74">
   <si>
     <t>Variable</t>
   </si>
@@ -258,6 +258,12 @@
   </si>
   <si>
     <t>Surrogate_sig</t>
+  </si>
+  <si>
+    <t>Graph?</t>
+  </si>
+  <si>
+    <t>test</t>
   </si>
 </sst>
 </file>
@@ -2480,17 +2486,18 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4796A85C-8317-4493-888D-443234A7E4BB}">
-  <dimension ref="A1:F104"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="16.81640625" customWidth="1"/>
-    <col min="3" max="3" width="19.6328125" customWidth="1"/>
-    <col min="4" max="4" width="19.36328125" customWidth="1"/>
-    <col min="5" max="5" width="17.453125" customWidth="1"/>
+    <col min="3" max="3" width="12.08984375" customWidth="1"/>
+    <col min="4" max="4" width="10.6328125" customWidth="1"/>
+    <col min="5" max="5" width="7.08984375" customWidth="1"/>
     <col min="6" max="6" width="15.08984375" customWidth="1"/>
+    <col min="7" max="7" width="15.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>61</v>
       </c>
@@ -2509,8 +2516,11 @@
       <c r="F1" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>64</v>
       </c>
@@ -2529,8 +2539,11 @@
       <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>64</v>
       </c>
@@ -2547,7 +2560,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>64</v>
       </c>
@@ -2564,7 +2577,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>64</v>
       </c>
@@ -2583,8 +2596,11 @@
       <c r="F5" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G5" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>64</v>
       </c>
@@ -2603,8 +2619,11 @@
       <c r="F6" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G6" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>64</v>
       </c>
@@ -2623,8 +2642,11 @@
       <c r="F7" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G7" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>64</v>
       </c>
@@ -2641,7 +2663,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>64</v>
       </c>
@@ -2660,8 +2682,11 @@
       <c r="F9" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G9" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>64</v>
       </c>
@@ -2678,7 +2703,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>64</v>
       </c>
@@ -2697,8 +2722,11 @@
       <c r="F11" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G11" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>64</v>
       </c>
@@ -2715,7 +2743,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>64</v>
       </c>
@@ -2732,7 +2760,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>64</v>
       </c>
@@ -2751,8 +2779,11 @@
       <c r="F14" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G14" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>64</v>
       </c>
@@ -2769,7 +2800,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>64</v>
       </c>
@@ -2788,8 +2819,11 @@
       <c r="F16" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G16" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>64</v>
       </c>
@@ -2808,8 +2842,11 @@
       <c r="F17" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G17" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>64</v>
       </c>
@@ -2826,7 +2863,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>64</v>
       </c>
@@ -2845,8 +2882,11 @@
       <c r="F19" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G19" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>64</v>
       </c>
@@ -2865,8 +2905,11 @@
       <c r="F20" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G20" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>64</v>
       </c>
@@ -2883,7 +2926,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>64</v>
       </c>
@@ -2902,8 +2945,11 @@
       <c r="F22" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G22" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>64</v>
       </c>
@@ -2922,8 +2968,11 @@
       <c r="F23" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G23" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>64</v>
       </c>
@@ -2940,7 +2989,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>64</v>
       </c>
@@ -2959,8 +3008,11 @@
       <c r="F25" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G25" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>64</v>
       </c>
@@ -2979,8 +3031,11 @@
       <c r="F26" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G26" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>64</v>
       </c>
@@ -2999,8 +3054,11 @@
       <c r="F27" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G27" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>64</v>
       </c>
@@ -3019,8 +3077,11 @@
       <c r="F28" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G28" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>4</v>
       </c>
@@ -3037,7 +3098,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>4</v>
       </c>
@@ -3054,7 +3115,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>4</v>
       </c>
@@ -3071,7 +3132,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>4</v>
       </c>
@@ -3090,8 +3151,11 @@
       <c r="F32" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G32" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>4</v>
       </c>
@@ -3108,7 +3172,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>4</v>
       </c>
@@ -3125,7 +3189,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>4</v>
       </c>
@@ -3144,8 +3208,11 @@
       <c r="F35" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G35" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>4</v>
       </c>
@@ -3164,8 +3231,11 @@
       <c r="F36" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G36" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>4</v>
       </c>
@@ -3184,8 +3254,11 @@
       <c r="F37" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G37" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>4</v>
       </c>
@@ -3202,7 +3275,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>4</v>
       </c>
@@ -3219,7 +3292,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="40" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>4</v>
       </c>
@@ -3238,8 +3311,11 @@
       <c r="F40" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G40" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>4</v>
       </c>
@@ -3258,8 +3334,11 @@
       <c r="F41" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G41" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>4</v>
       </c>
@@ -3278,8 +3357,11 @@
       <c r="F42" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G42" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>4</v>
       </c>
@@ -3296,7 +3378,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>4</v>
       </c>
@@ -3313,7 +3395,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="45" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>4</v>
       </c>
@@ -3332,8 +3414,11 @@
       <c r="F45" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G45" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>4</v>
       </c>
@@ -3350,7 +3435,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>4</v>
       </c>
@@ -3367,7 +3452,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="48" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>4</v>
       </c>
@@ -3386,8 +3471,11 @@
       <c r="F48" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G48" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>4</v>
       </c>
@@ -3404,7 +3492,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>4</v>
       </c>
@@ -3421,7 +3509,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="51" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>4</v>
       </c>
@@ -3440,8 +3528,11 @@
       <c r="F51" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G51" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>4</v>
       </c>
@@ -3458,7 +3549,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>4</v>
       </c>
@@ -3475,7 +3566,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>4</v>
       </c>
@@ -3492,7 +3583,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>4</v>
       </c>
@@ -3509,7 +3600,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="56" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>46</v>
       </c>
@@ -3525,8 +3616,14 @@
       <c r="E56" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="F56" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>46</v>
       </c>
@@ -3542,8 +3639,14 @@
       <c r="E57" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="F57" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>46</v>
       </c>
@@ -3560,7 +3663,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>46</v>
       </c>
@@ -3577,7 +3680,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>46</v>
       </c>
@@ -3594,7 +3697,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>46</v>
       </c>
@@ -3611,7 +3714,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>46</v>
       </c>
@@ -3628,7 +3731,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>46</v>
       </c>
@@ -3645,7 +3748,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="64" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>46</v>
       </c>
@@ -3661,8 +3764,14 @@
       <c r="E64" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="F64" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>46</v>
       </c>
@@ -3678,8 +3787,14 @@
       <c r="E65" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="F65" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>46</v>
       </c>
@@ -3695,8 +3810,14 @@
       <c r="E66" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F66" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>46</v>
       </c>
@@ -3713,7 +3834,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>46</v>
       </c>
@@ -3730,7 +3851,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>46</v>
       </c>
@@ -3747,7 +3868,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>46</v>
       </c>
@@ -3764,7 +3885,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>46</v>
       </c>
@@ -3781,7 +3902,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>46</v>
       </c>
@@ -3798,7 +3919,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>46</v>
       </c>
@@ -3814,8 +3935,14 @@
       <c r="E73" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F73" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>46</v>
       </c>
@@ -3832,7 +3959,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>46</v>
       </c>
@@ -3849,7 +3976,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>46</v>
       </c>
@@ -3866,7 +3993,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>46</v>
       </c>
@@ -3883,7 +4010,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>58</v>
       </c>
@@ -3900,7 +4027,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>58</v>
       </c>
@@ -3917,7 +4044,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>58</v>
       </c>
@@ -3934,7 +4061,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>58</v>
       </c>
@@ -3951,7 +4078,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>58</v>
       </c>
@@ -3968,7 +4095,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>58</v>
       </c>
@@ -3985,7 +4112,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="84" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>58</v>
       </c>
@@ -4004,8 +4131,11 @@
       <c r="F84" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G84" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>58</v>
       </c>
@@ -4022,7 +4152,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="86" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>58</v>
       </c>
@@ -4041,8 +4171,11 @@
       <c r="F86" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G86" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>58</v>
       </c>
@@ -4059,7 +4192,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>58</v>
       </c>
@@ -4076,7 +4209,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="89" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>58</v>
       </c>
@@ -4095,8 +4228,11 @@
       <c r="F89" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="90" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G89" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>58</v>
       </c>
@@ -4115,8 +4251,11 @@
       <c r="F90" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G90" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>58</v>
       </c>
@@ -4135,8 +4274,11 @@
       <c r="F91" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G91" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>58</v>
       </c>
@@ -4153,7 +4295,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>58</v>
       </c>
@@ -4170,7 +4312,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>58</v>
       </c>
@@ -4187,7 +4329,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>58</v>
       </c>
@@ -4204,7 +4346,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>58</v>
       </c>
@@ -4221,7 +4363,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>58</v>
       </c>
@@ -4238,7 +4380,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="98" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>58</v>
       </c>
@@ -4257,8 +4399,11 @@
       <c r="F98" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G98" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>58</v>
       </c>
@@ -4275,7 +4420,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>58</v>
       </c>
@@ -4292,7 +4437,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="101" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>58</v>
       </c>
@@ -4311,8 +4456,11 @@
       <c r="F101" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="102" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G101" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>58</v>
       </c>
@@ -4331,8 +4479,11 @@
       <c r="F102" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="103" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="G102" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>58</v>
       </c>
@@ -4351,8 +4502,11 @@
       <c r="F103" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G103" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
adding in cumulative flows
</commit_message>
<xml_diff>
--- a/parameters_CCM.xlsx
+++ b/parameters_CCM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b94c59a01e372ca2/Desktop/Algal_blooms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="781" documentId="8_{A267BACA-5322-4D14-AD98-2B8644D6D7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C36811B-19E7-478D-8061-DECCF14C2683}"/>
+  <xr:revisionPtr revIDLastSave="791" documentId="8_{A267BACA-5322-4D14-AD98-2B8644D6D7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66DA1EF5-DC6E-4BA9-8D87-E08D7AACF0F8}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" activeTab="6" xr2:uid="{96C955FB-9A51-4D0B-AF49-129559A448B6}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{96C955FB-9A51-4D0B-AF49-129559A448B6}"/>
   </bookViews>
   <sheets>
     <sheet name="Run1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="76">
   <si>
     <t>Variable</t>
   </si>
@@ -264,6 +264,12 @@
   </si>
   <si>
     <t>test</t>
+  </si>
+  <si>
+    <t>aflow_cum</t>
+  </si>
+  <si>
+    <t>mflow_cum</t>
   </si>
 </sst>
 </file>
@@ -1741,7 +1747,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0219A31A-9904-40E1-98EE-E1AAB97C02AB}">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.08984375" customWidth="1"/>
@@ -2265,6 +2271,40 @@
         <v>6</v>
       </c>
       <c r="F30" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B31" s="1">
+        <v>3</v>
+      </c>
+      <c r="C31" s="1">
+        <v>3</v>
+      </c>
+      <c r="D31" s="1">
+        <v>3</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B32" s="1">
+        <v>3</v>
+      </c>
+      <c r="C32" s="1">
+        <v>3</v>
+      </c>
+      <c r="D32" s="1">
+        <v>3</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dead creak EDM from sentinel-2 imagery
</commit_message>
<xml_diff>
--- a/parameters_CCM.xlsx
+++ b/parameters_CCM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rodemann/Algal_EDM/Algal_blooms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D4EF0AE-37A3-7545-93DE-C6F0ADAC0D42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E677FB-D1CF-5445-A9BB-28B136E503EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="6" xr2:uid="{96C955FB-9A51-4D0B-AF49-129559A448B6}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="906" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="936" uniqueCount="99">
   <si>
     <t>Variable</t>
   </si>
@@ -332,6 +332,12 @@
   </si>
   <si>
     <t>echl</t>
+  </si>
+  <si>
+    <t>dcbr</t>
+  </si>
+  <si>
+    <t>dcbre</t>
   </si>
 </sst>
 </file>
@@ -1816,7 +1822,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0219A31A-9904-40E1-98EE-E1AAB97C02AB}">
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.1640625" customWidth="1"/>
@@ -2725,6 +2731,40 @@
       </c>
       <c r="E53" s="1" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B54" s="1">
+        <v>2</v>
+      </c>
+      <c r="C54" s="1">
+        <v>4</v>
+      </c>
+      <c r="D54" s="1">
+        <v>2</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B55" s="1">
+        <v>5</v>
+      </c>
+      <c r="C55" s="1">
+        <v>4</v>
+      </c>
+      <c r="D55" s="1">
+        <v>4</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -2945,7 +2985,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4796A85C-8317-4493-888D-443234A7E4BB}">
-  <dimension ref="A1:G168"/>
+  <dimension ref="A1:G174"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="16.83203125" customWidth="1"/>
@@ -3956,38 +3996,50 @@
         <v>21</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>4</v>
-      </c>
-      <c r="B51" t="s">
-        <v>11</v>
-      </c>
-      <c r="C51">
-        <v>0.111</v>
-      </c>
-      <c r="D51">
-        <v>-12</v>
-      </c>
-      <c r="E51" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>4</v>
-      </c>
-      <c r="B52" t="s">
-        <v>7</v>
-      </c>
-      <c r="C52">
-        <v>0.38</v>
-      </c>
-      <c r="D52">
-        <v>-12</v>
-      </c>
-      <c r="E52" t="s">
-        <v>21</v>
+    <row r="51" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C51" s="1">
+        <v>0.32400000000000001</v>
+      </c>
+      <c r="D51" s="1">
+        <v>-11</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C52" s="1">
+        <v>0.45300000000000001</v>
+      </c>
+      <c r="D52" s="1">
+        <v>-10</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
@@ -3995,10 +4047,10 @@
         <v>4</v>
       </c>
       <c r="B53" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C53">
-        <v>0.28499999999999998</v>
+        <v>0.111</v>
       </c>
       <c r="D53">
         <v>-12</v>
@@ -4007,27 +4059,21 @@
         <v>21</v>
       </c>
     </row>
-    <row r="54" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C54" s="1">
-        <v>0.33300000000000002</v>
-      </c>
-      <c r="D54" s="1">
-        <v>6</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>72</v>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>4</v>
+      </c>
+      <c r="B54" t="s">
+        <v>7</v>
+      </c>
+      <c r="C54">
+        <v>0.38</v>
+      </c>
+      <c r="D54">
+        <v>-12</v>
+      </c>
+      <c r="E54" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
@@ -4035,79 +4081,73 @@
         <v>4</v>
       </c>
       <c r="B55" t="s">
+        <v>8</v>
+      </c>
+      <c r="C55">
+        <v>0.28499999999999998</v>
+      </c>
+      <c r="D55">
+        <v>-12</v>
+      </c>
+      <c r="E55" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C56" s="1">
+        <v>0.33300000000000002</v>
+      </c>
+      <c r="D56" s="1">
+        <v>6</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>4</v>
+      </c>
+      <c r="B57" t="s">
         <v>31</v>
       </c>
-      <c r="C55">
+      <c r="C57">
         <v>0.16800000000000001</v>
       </c>
-      <c r="D55">
+      <c r="D57">
         <v>5</v>
       </c>
-      <c r="E55" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>4</v>
-      </c>
-      <c r="B56" t="s">
+      <c r="E57" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>4</v>
+      </c>
+      <c r="B58" t="s">
         <v>68</v>
       </c>
-      <c r="C56">
+      <c r="C58">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="D56">
-        <v>2</v>
-      </c>
-      <c r="E56" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C57" s="1">
-        <v>0.223</v>
-      </c>
-      <c r="D57" s="1">
-        <v>-4</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C58" s="1">
-        <v>0.47</v>
-      </c>
-      <c r="D58" s="1">
-        <v>-4</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>6</v>
+      <c r="D58">
+        <v>2</v>
+      </c>
+      <c r="E58" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="59" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -4115,102 +4155,102 @@
         <v>4</v>
       </c>
       <c r="B59" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C59" s="1">
+        <v>0.223</v>
+      </c>
+      <c r="D59" s="1">
+        <v>-4</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C60" s="1">
+        <v>0.47</v>
+      </c>
+      <c r="D60" s="1">
+        <v>-4</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C59" s="1">
+      <c r="C61" s="1">
         <v>0.6</v>
       </c>
-      <c r="D59" s="1">
+      <c r="D61" s="1">
         <v>7</v>
       </c>
-      <c r="E59" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G59" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>4</v>
-      </c>
-      <c r="B60" t="s">
+      <c r="E61" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>4</v>
+      </c>
+      <c r="B62" t="s">
         <v>28</v>
       </c>
-      <c r="C60">
+      <c r="C62">
         <v>0.192</v>
       </c>
-      <c r="D60">
+      <c r="D62">
         <v>5</v>
       </c>
-      <c r="E60" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
-        <v>4</v>
-      </c>
-      <c r="B61" t="s">
+      <c r="E62" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>4</v>
+      </c>
+      <c r="B63" t="s">
         <v>27</v>
       </c>
-      <c r="C61">
+      <c r="C63">
         <v>-0.154</v>
       </c>
-      <c r="D61">
+      <c r="D63">
         <v>9</v>
       </c>
-      <c r="E61" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C62" s="1">
-        <v>0.496</v>
-      </c>
-      <c r="D62" s="1">
-        <v>-8</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C63" s="1">
-        <v>0.45600000000000002</v>
-      </c>
-      <c r="D63" s="1">
-        <v>8</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G63" s="1" t="s">
-        <v>6</v>
+      <c r="E63" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="64" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -4218,78 +4258,84 @@
         <v>4</v>
       </c>
       <c r="B64" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C64" s="1">
+        <v>0.496</v>
+      </c>
+      <c r="D64" s="1">
+        <v>-8</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C65" s="1">
+        <v>0.45600000000000002</v>
+      </c>
+      <c r="D65" s="1">
+        <v>8</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B66" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C64" s="1">
+      <c r="C66" s="1">
         <v>0.73</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D66" s="1">
         <v>-10</v>
       </c>
-      <c r="E64" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F64" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G64" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>4</v>
-      </c>
-      <c r="B65" t="s">
+      <c r="E66" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>4</v>
+      </c>
+      <c r="B67" t="s">
         <v>59</v>
       </c>
-      <c r="C65">
+      <c r="C67">
         <v>-0.13600000000000001</v>
       </c>
-      <c r="D65">
+      <c r="D67">
         <v>9</v>
       </c>
-      <c r="E65" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
-        <v>4</v>
-      </c>
-      <c r="B66" t="s">
-        <v>53</v>
-      </c>
-      <c r="C66">
-        <v>0.39800000000000002</v>
-      </c>
-      <c r="D66">
-        <v>9</v>
-      </c>
-      <c r="E66" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C67" s="1">
-        <v>0.503</v>
-      </c>
-      <c r="D67" s="1">
-        <v>-12</v>
-      </c>
-      <c r="E67" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F67" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G67" s="1" t="s">
+      <c r="E67" t="s">
         <v>21</v>
       </c>
     </row>
@@ -4298,55 +4344,55 @@
         <v>4</v>
       </c>
       <c r="B68" t="s">
+        <v>53</v>
+      </c>
+      <c r="C68">
+        <v>0.39800000000000002</v>
+      </c>
+      <c r="D68">
+        <v>9</v>
+      </c>
+      <c r="E68" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C69" s="1">
+        <v>0.503</v>
+      </c>
+      <c r="D69" s="1">
+        <v>-12</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>4</v>
+      </c>
+      <c r="B70" t="s">
         <v>55</v>
       </c>
-      <c r="C68">
+      <c r="C70">
         <v>0.313</v>
       </c>
-      <c r="D68">
+      <c r="D70">
         <v>7</v>
       </c>
-      <c r="E68" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
-        <v>4</v>
-      </c>
-      <c r="B69" t="s">
-        <v>56</v>
-      </c>
-      <c r="C69">
-        <v>0.24099999999999999</v>
-      </c>
-      <c r="D69">
-        <v>5</v>
-      </c>
-      <c r="E69" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C70" s="1">
-        <v>0.29199999999999998</v>
-      </c>
-      <c r="D70" s="1">
-        <v>1</v>
-      </c>
-      <c r="E70" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F70" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G70" s="1" t="s">
+      <c r="E70" t="s">
         <v>21</v>
       </c>
     </row>
@@ -4355,56 +4401,56 @@
         <v>4</v>
       </c>
       <c r="B71" t="s">
+        <v>56</v>
+      </c>
+      <c r="C71">
+        <v>0.24099999999999999</v>
+      </c>
+      <c r="D71">
+        <v>5</v>
+      </c>
+      <c r="E71" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C72" s="1">
+        <v>0.29199999999999998</v>
+      </c>
+      <c r="D72" s="1">
+        <v>1</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>4</v>
+      </c>
+      <c r="B73" t="s">
         <v>58</v>
       </c>
-      <c r="C71">
+      <c r="C73">
         <v>-4.0000000000000001E-3</v>
       </c>
-      <c r="D71">
+      <c r="D73">
         <v>-1</v>
       </c>
-      <c r="E71" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
-        <v>4</v>
-      </c>
-      <c r="B72" t="s">
-        <v>24</v>
-      </c>
-      <c r="C72">
-        <v>0.25900000000000001</v>
-      </c>
-      <c r="D72">
-        <v>-5</v>
-      </c>
-      <c r="E72" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C73" s="1">
-        <v>0.63600000000000001</v>
-      </c>
-      <c r="D73" s="1">
-        <v>7</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G73" s="1" t="s">
-        <v>6</v>
+      <c r="E73" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.2">
@@ -4412,33 +4458,39 @@
         <v>4</v>
       </c>
       <c r="B74" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C74">
-        <v>5.8999999999999997E-2</v>
+        <v>0.25900000000000001</v>
       </c>
       <c r="D74">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="E74" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
-        <v>4</v>
-      </c>
-      <c r="B75" t="s">
-        <v>33</v>
-      </c>
-      <c r="C75">
-        <v>0.32900000000000001</v>
-      </c>
-      <c r="D75">
-        <v>-4</v>
-      </c>
-      <c r="E75" t="s">
-        <v>21</v>
+    <row r="75" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C75" s="1">
+        <v>0.63600000000000001</v>
+      </c>
+      <c r="D75" s="1">
+        <v>7</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
@@ -4446,10 +4498,10 @@
         <v>4</v>
       </c>
       <c r="B76" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="C76">
-        <v>6.7000000000000004E-2</v>
+        <v>5.8999999999999997E-2</v>
       </c>
       <c r="D76">
         <v>0</v>
@@ -4463,106 +4515,106 @@
         <v>4</v>
       </c>
       <c r="B77" t="s">
+        <v>33</v>
+      </c>
+      <c r="C77">
+        <v>0.32900000000000001</v>
+      </c>
+      <c r="D77">
+        <v>-4</v>
+      </c>
+      <c r="E77" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>4</v>
+      </c>
+      <c r="B78" t="s">
+        <v>34</v>
+      </c>
+      <c r="C78">
+        <v>6.7000000000000004E-2</v>
+      </c>
+      <c r="D78">
+        <v>0</v>
+      </c>
+      <c r="E78" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>4</v>
+      </c>
+      <c r="B79" t="s">
         <v>69</v>
       </c>
-      <c r="C77">
+      <c r="C79">
         <v>-3.3000000000000002E-2</v>
       </c>
-      <c r="D77">
-        <v>4</v>
-      </c>
-      <c r="E77" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B78" s="1" t="s">
+      <c r="D79">
+        <v>4</v>
+      </c>
+      <c r="E79" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B80" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C78" s="1">
+      <c r="C80" s="1">
         <v>0.14000000000000001</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D80" s="1">
         <v>-2</v>
       </c>
-      <c r="E78" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F78" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G78" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B79" s="2" t="s">
+      <c r="E80" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B81" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C79" s="2">
+      <c r="C81" s="2">
         <v>0.161</v>
       </c>
-      <c r="D79" s="2">
+      <c r="D81" s="2">
         <v>8</v>
       </c>
-      <c r="E79" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A80" t="s">
-        <v>4</v>
-      </c>
-      <c r="B80" s="2" t="s">
+      <c r="E81" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>4</v>
+      </c>
+      <c r="B82" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C80">
+      <c r="C82">
         <v>0</v>
       </c>
-      <c r="D80">
+      <c r="D82">
         <v>0</v>
       </c>
-      <c r="E80" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
-        <v>4</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C81">
-        <v>0</v>
-      </c>
-      <c r="D81">
-        <v>0</v>
-      </c>
-      <c r="E81" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C82" s="2">
-        <v>0</v>
-      </c>
-      <c r="D82" s="2">
-        <v>0</v>
-      </c>
-      <c r="E82" s="2" t="s">
+      <c r="E82" t="s">
         <v>21</v>
       </c>
     </row>
@@ -4571,7 +4623,7 @@
         <v>4</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C83">
         <v>0</v>
@@ -4588,13 +4640,13 @@
         <v>4</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C84" s="2">
-        <v>0.245</v>
+        <v>0</v>
       </c>
       <c r="D84" s="2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>21</v>
@@ -4605,7 +4657,7 @@
         <v>4</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C85">
         <v>0</v>
@@ -4617,18 +4669,18 @@
         <v>21</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
+    <row r="86" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A86" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C86" s="2">
-        <v>8.8999999999999996E-2</v>
+        <v>0.245</v>
       </c>
       <c r="D86" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>21</v>
@@ -4639,49 +4691,49 @@
         <v>4</v>
       </c>
       <c r="B87" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C87">
+        <v>0</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>4</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C88" s="2">
+        <v>8.8999999999999996E-2</v>
+      </c>
+      <c r="D88" s="2">
+        <v>7</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>4</v>
+      </c>
+      <c r="B89" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C87">
+      <c r="C89">
         <v>8.6999999999999994E-2</v>
       </c>
-      <c r="D87">
+      <c r="D89">
         <v>-9</v>
       </c>
-      <c r="E87" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A88" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C88" s="2">
-        <v>0.11700000000000001</v>
-      </c>
-      <c r="D88" s="2">
-        <v>12</v>
-      </c>
-      <c r="E88" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B89" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C89" s="2">
-        <v>0.215</v>
-      </c>
-      <c r="D89" s="2">
-        <v>9</v>
-      </c>
-      <c r="E89" s="2" t="s">
+      <c r="E89" t="s">
         <v>21</v>
       </c>
     </row>
@@ -4690,13 +4742,13 @@
         <v>4</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C90" s="2">
-        <v>0.13300000000000001</v>
+        <v>0.11700000000000001</v>
       </c>
       <c r="D90" s="2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>21</v>
@@ -4707,13 +4759,13 @@
         <v>4</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C91" s="2">
-        <v>7.3999999999999996E-2</v>
+        <v>0.215</v>
       </c>
       <c r="D91" s="2">
-        <v>-4</v>
+        <v>9</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>21</v>
@@ -4724,13 +4776,13 @@
         <v>4</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C92" s="2">
-        <v>0.254</v>
+        <v>0.13300000000000001</v>
       </c>
       <c r="D92" s="2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>21</v>
@@ -4741,13 +4793,13 @@
         <v>4</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C93" s="2">
-        <v>0.217</v>
+        <v>7.3999999999999996E-2</v>
       </c>
       <c r="D93" s="2">
-        <v>8</v>
+        <v>-4</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>21</v>
@@ -4758,13 +4810,13 @@
         <v>4</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C94" s="2">
-        <v>0.14799999999999999</v>
+        <v>0.254</v>
       </c>
       <c r="D94" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E94" s="2" t="s">
         <v>21</v>
@@ -4775,13 +4827,13 @@
         <v>4</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C95" s="2">
-        <v>0</v>
+        <v>0.217</v>
       </c>
       <c r="D95" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>21</v>
@@ -4792,10 +4844,10 @@
         <v>4</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C96" s="2">
-        <v>0.33</v>
+        <v>0.14799999999999999</v>
       </c>
       <c r="D96" s="2">
         <v>9</v>
@@ -4809,13 +4861,13 @@
         <v>4</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C97" s="2">
-        <v>0.29099999999999998</v>
+        <v>0</v>
       </c>
       <c r="D97" s="2">
-        <v>-9</v>
+        <v>0</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>21</v>
@@ -4826,130 +4878,130 @@
         <v>4</v>
       </c>
       <c r="B98" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C98" s="2">
+        <v>0.33</v>
+      </c>
+      <c r="D98" s="2">
+        <v>9</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A99" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C99" s="2">
+        <v>0.29099999999999998</v>
+      </c>
+      <c r="D99" s="2">
+        <v>-9</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A100" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B100" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C98" s="2">
+      <c r="C100" s="2">
         <v>0</v>
       </c>
-      <c r="D98" s="2">
+      <c r="D100" s="2">
         <v>0</v>
       </c>
-      <c r="E98" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A99" s="1" t="s">
+      <c r="E100" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A101" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C101" s="2">
+        <v>6.2E-2</v>
+      </c>
+      <c r="D101" s="2">
+        <v>-9</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A102" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C102" s="2">
+        <v>4.9000000000000002E-2</v>
+      </c>
+      <c r="D102" s="2">
+        <v>-12</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A103" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B99" s="1" t="s">
+      <c r="B103" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C99" s="1">
+      <c r="C103" s="1">
         <v>0.36299999999999999</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D103" s="1">
         <v>-7</v>
       </c>
-      <c r="E99" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F99" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G99" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A100" s="1" t="s">
+      <c r="E103" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G103" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A104" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B100" s="1" t="s">
+      <c r="B104" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C100" s="1">
+      <c r="C104" s="1">
         <v>0.38500000000000001</v>
       </c>
-      <c r="D100" s="1">
-        <v>6</v>
-      </c>
-      <c r="E100" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F100" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G100" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
-        <v>46</v>
-      </c>
-      <c r="B101" t="s">
-        <v>8</v>
-      </c>
-      <c r="C101">
-        <v>5.8000000000000003E-2</v>
-      </c>
-      <c r="D101">
-        <v>6</v>
-      </c>
-      <c r="E101" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
-        <v>46</v>
-      </c>
-      <c r="B102" t="s">
-        <v>12</v>
-      </c>
-      <c r="C102">
-        <v>8.6999999999999994E-2</v>
-      </c>
-      <c r="D102">
-        <v>-2</v>
-      </c>
-      <c r="E102" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A103" t="s">
-        <v>46</v>
-      </c>
-      <c r="B103" t="s">
-        <v>31</v>
-      </c>
-      <c r="C103">
-        <v>0.35</v>
-      </c>
-      <c r="D103">
-        <v>9</v>
-      </c>
-      <c r="E103" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A104" t="s">
-        <v>46</v>
-      </c>
-      <c r="B104" t="s">
-        <v>63</v>
-      </c>
-      <c r="C104">
-        <v>0.17199999999999999</v>
-      </c>
-      <c r="D104">
-        <v>-2</v>
-      </c>
-      <c r="E104" t="s">
-        <v>21</v>
+      <c r="D104" s="1">
+        <v>6</v>
+      </c>
+      <c r="E104" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F104" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G104" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.2">
@@ -4957,13 +5009,13 @@
         <v>46</v>
       </c>
       <c r="B105" t="s">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="C105">
-        <v>0.111</v>
+        <v>5.8000000000000003E-2</v>
       </c>
       <c r="D105">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E105" t="s">
         <v>21</v>
@@ -4974,10 +5026,10 @@
         <v>46</v>
       </c>
       <c r="B106" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="C106">
-        <v>0.191</v>
+        <v>8.6999999999999994E-2</v>
       </c>
       <c r="D106">
         <v>-2</v>
@@ -4986,72 +5038,54 @@
         <v>21</v>
       </c>
     </row>
-    <row r="107" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A107" s="1" t="s">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
         <v>46</v>
       </c>
-      <c r="B107" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C107" s="1">
-        <v>0.47699999999999998</v>
-      </c>
-      <c r="D107" s="1">
-        <v>6</v>
-      </c>
-      <c r="E107" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F107" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G107" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="108" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A108" s="1" t="s">
+      <c r="B107" t="s">
+        <v>31</v>
+      </c>
+      <c r="C107">
+        <v>0.35</v>
+      </c>
+      <c r="D107">
+        <v>9</v>
+      </c>
+      <c r="E107" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
         <v>46</v>
       </c>
-      <c r="B108" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C108" s="1">
-        <v>0.318</v>
-      </c>
-      <c r="D108" s="1">
-        <v>9</v>
-      </c>
-      <c r="E108" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F108" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G108" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="109" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A109" s="1" t="s">
+      <c r="B108" t="s">
+        <v>63</v>
+      </c>
+      <c r="C108">
+        <v>0.17199999999999999</v>
+      </c>
+      <c r="D108">
+        <v>-2</v>
+      </c>
+      <c r="E108" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
         <v>46</v>
       </c>
-      <c r="B109" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C109" s="1">
-        <v>0.51800000000000002</v>
-      </c>
-      <c r="D109" s="1">
-        <v>7</v>
-      </c>
-      <c r="E109" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F109" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G109" s="1" t="s">
+      <c r="B109" t="s">
+        <v>68</v>
+      </c>
+      <c r="C109">
+        <v>0.111</v>
+      </c>
+      <c r="D109">
+        <v>12</v>
+      </c>
+      <c r="E109" t="s">
         <v>21</v>
       </c>
     </row>
@@ -5060,66 +5094,84 @@
         <v>46</v>
       </c>
       <c r="B110" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="C110">
-        <v>0.121</v>
+        <v>0.191</v>
       </c>
       <c r="D110">
-        <v>-12</v>
+        <v>-2</v>
       </c>
       <c r="E110" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A111" t="s">
+    <row r="111" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A111" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B111" t="s">
-        <v>53</v>
-      </c>
-      <c r="C111">
-        <v>0.36299999999999999</v>
-      </c>
-      <c r="D111">
-        <v>8</v>
-      </c>
-      <c r="E111" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A112" t="s">
+      <c r="B111" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C111" s="1">
+        <v>0.47699999999999998</v>
+      </c>
+      <c r="D111" s="1">
+        <v>6</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G111" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A112" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B112" t="s">
-        <v>50</v>
-      </c>
-      <c r="C112">
-        <v>0.221</v>
-      </c>
-      <c r="D112">
-        <v>1</v>
-      </c>
-      <c r="E112" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A113" t="s">
+      <c r="B112" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C112" s="1">
+        <v>0.318</v>
+      </c>
+      <c r="D112" s="1">
+        <v>9</v>
+      </c>
+      <c r="E112" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G112" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A113" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B113" t="s">
-        <v>55</v>
-      </c>
-      <c r="C113">
-        <v>0.14399999999999999</v>
-      </c>
-      <c r="D113">
-        <v>12</v>
-      </c>
-      <c r="E113" t="s">
+      <c r="B113" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C113" s="1">
+        <v>0.51800000000000002</v>
+      </c>
+      <c r="D113" s="1">
+        <v>7</v>
+      </c>
+      <c r="E113" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G113" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -5128,13 +5180,13 @@
         <v>46</v>
       </c>
       <c r="B114" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C114">
-        <v>0.189</v>
+        <v>0.121</v>
       </c>
       <c r="D114">
-        <v>-2</v>
+        <v>-12</v>
       </c>
       <c r="E114" t="s">
         <v>21</v>
@@ -5145,39 +5197,33 @@
         <v>46</v>
       </c>
       <c r="B115" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C115">
-        <v>0.04</v>
+        <v>0.36299999999999999</v>
       </c>
       <c r="D115">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E115" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="116" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A116" s="1" t="s">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
         <v>46</v>
       </c>
-      <c r="B116" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C116" s="1">
-        <v>0.38400000000000001</v>
-      </c>
-      <c r="D116" s="1">
-        <v>-3</v>
-      </c>
-      <c r="E116" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F116" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G116" s="1" t="s">
-        <v>6</v>
+      <c r="B116" t="s">
+        <v>50</v>
+      </c>
+      <c r="C116">
+        <v>0.221</v>
+      </c>
+      <c r="D116">
+        <v>1</v>
+      </c>
+      <c r="E116" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.2">
@@ -5185,13 +5231,13 @@
         <v>46</v>
       </c>
       <c r="B117" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="C117">
-        <v>0.23</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="D117">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E117" t="s">
         <v>21</v>
@@ -5202,13 +5248,13 @@
         <v>46</v>
       </c>
       <c r="B118" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="C118">
-        <v>0.255</v>
+        <v>0.189</v>
       </c>
       <c r="D118">
-        <v>4</v>
+        <v>-2</v>
       </c>
       <c r="E118" t="s">
         <v>21</v>
@@ -5219,10 +5265,10 @@
         <v>46</v>
       </c>
       <c r="B119" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="C119">
-        <v>2.8000000000000001E-2</v>
+        <v>0.04</v>
       </c>
       <c r="D119">
         <v>4</v>
@@ -5231,35 +5277,41 @@
         <v>21</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A120" t="s">
+    <row r="120" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A120" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B120" t="s">
-        <v>69</v>
-      </c>
-      <c r="C120">
-        <v>0.26600000000000001</v>
-      </c>
-      <c r="D120">
-        <v>-11</v>
-      </c>
-      <c r="E120" t="s">
-        <v>21</v>
+      <c r="B120" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C120" s="1">
+        <v>0.38400000000000001</v>
+      </c>
+      <c r="D120" s="1">
+        <v>-3</v>
+      </c>
+      <c r="E120" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F120" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G120" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="B121" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="C121">
-        <v>8.1000000000000003E-2</v>
+        <v>0.23</v>
       </c>
       <c r="D121">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E121" t="s">
         <v>21</v>
@@ -5267,16 +5319,16 @@
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="B122" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="C122">
-        <v>2.1999999999999999E-2</v>
+        <v>0.255</v>
       </c>
       <c r="D122">
-        <v>-10</v>
+        <v>4</v>
       </c>
       <c r="E122" t="s">
         <v>21</v>
@@ -5284,16 +5336,16 @@
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="B123" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="C123">
-        <v>2.9000000000000001E-2</v>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="D123">
-        <v>-3</v>
+        <v>4</v>
       </c>
       <c r="E123" t="s">
         <v>21</v>
@@ -5301,16 +5353,16 @@
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="B124" t="s">
-        <v>12</v>
+        <v>69</v>
       </c>
       <c r="C124">
-        <v>0.23300000000000001</v>
+        <v>0.26600000000000001</v>
       </c>
       <c r="D124">
-        <v>2</v>
+        <v>-11</v>
       </c>
       <c r="E124" t="s">
         <v>21</v>
@@ -5321,13 +5373,13 @@
         <v>58</v>
       </c>
       <c r="B125" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="C125">
-        <v>0.20200000000000001</v>
+        <v>8.1000000000000003E-2</v>
       </c>
       <c r="D125">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E125" t="s">
         <v>21</v>
@@ -5338,39 +5390,33 @@
         <v>58</v>
       </c>
       <c r="B126" t="s">
-        <v>68</v>
+        <v>7</v>
       </c>
       <c r="C126">
-        <v>0.36499999999999999</v>
+        <v>2.1999999999999999E-2</v>
       </c>
       <c r="D126">
-        <v>11</v>
+        <v>-10</v>
       </c>
       <c r="E126" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="127" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A127" s="1" t="s">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
         <v>58</v>
       </c>
-      <c r="B127" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C127" s="1">
-        <v>0.61799999999999999</v>
-      </c>
-      <c r="D127" s="1">
-        <v>-6</v>
-      </c>
-      <c r="E127" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F127" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G127" s="1" t="s">
-        <v>6</v>
+      <c r="B127" t="s">
+        <v>8</v>
+      </c>
+      <c r="C127">
+        <v>2.9000000000000001E-2</v>
+      </c>
+      <c r="D127">
+        <v>-3</v>
+      </c>
+      <c r="E127" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.2">
@@ -5378,39 +5424,33 @@
         <v>58</v>
       </c>
       <c r="B128" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C128">
-        <v>0.20699999999999999</v>
+        <v>0.23300000000000001</v>
       </c>
       <c r="D128">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E128" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="129" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A129" s="1" t="s">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A129" t="s">
         <v>58</v>
       </c>
-      <c r="B129" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C129" s="1">
-        <v>0.35399999999999998</v>
-      </c>
-      <c r="D129" s="1">
+      <c r="B129" t="s">
+        <v>31</v>
+      </c>
+      <c r="C129">
+        <v>0.20200000000000001</v>
+      </c>
+      <c r="D129">
         <v>1</v>
       </c>
-      <c r="E129" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F129" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G129" s="1" t="s">
-        <v>6</v>
+      <c r="E129" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.2">
@@ -5418,56 +5458,56 @@
         <v>58</v>
       </c>
       <c r="B130" t="s">
-        <v>28</v>
+        <v>68</v>
       </c>
       <c r="C130">
-        <v>0.193</v>
+        <v>0.36499999999999999</v>
       </c>
       <c r="D130">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E130" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A131" t="s">
+    <row r="131" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A131" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B131" t="s">
-        <v>27</v>
-      </c>
-      <c r="C131">
-        <v>0.02</v>
-      </c>
-      <c r="D131">
-        <v>8</v>
-      </c>
-      <c r="E131" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="132" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A132" s="1" t="s">
+      <c r="B131" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C131" s="1">
+        <v>0.61799999999999999</v>
+      </c>
+      <c r="D131" s="1">
+        <v>-6</v>
+      </c>
+      <c r="E131" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F131" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G131" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A132" t="s">
         <v>58</v>
       </c>
-      <c r="B132" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C132" s="1">
-        <v>0.40699999999999997</v>
-      </c>
-      <c r="D132" s="1">
-        <v>-11</v>
-      </c>
-      <c r="E132" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F132" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G132" s="1" t="s">
-        <v>6</v>
+      <c r="B132" t="s">
+        <v>22</v>
+      </c>
+      <c r="C132">
+        <v>0.20699999999999999</v>
+      </c>
+      <c r="D132">
+        <v>5</v>
+      </c>
+      <c r="E132" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="133" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -5475,13 +5515,13 @@
         <v>58</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C133" s="1">
-        <v>0.27400000000000002</v>
+        <v>0.35399999999999998</v>
       </c>
       <c r="D133" s="1">
-        <v>-9</v>
+        <v>1</v>
       </c>
       <c r="E133" s="1" t="s">
         <v>6</v>
@@ -5493,27 +5533,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="134" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A134" s="1" t="s">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A134" t="s">
         <v>58</v>
       </c>
-      <c r="B134" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C134" s="1">
-        <v>0.35</v>
-      </c>
-      <c r="D134" s="1">
-        <v>-10</v>
-      </c>
-      <c r="E134" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F134" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G134" s="1" t="s">
-        <v>6</v>
+      <c r="B134" t="s">
+        <v>28</v>
+      </c>
+      <c r="C134">
+        <v>0.193</v>
+      </c>
+      <c r="D134">
+        <v>0</v>
+      </c>
+      <c r="E134" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.2">
@@ -5521,67 +5555,85 @@
         <v>58</v>
       </c>
       <c r="B135" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="C135">
-        <v>0.13100000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="D135">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E135" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A136" t="s">
+    <row r="136" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A136" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B136" t="s">
-        <v>53</v>
-      </c>
-      <c r="C136">
-        <v>0.33800000000000002</v>
-      </c>
-      <c r="D136">
+      <c r="B136" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C136" s="1">
+        <v>0.40699999999999997</v>
+      </c>
+      <c r="D136" s="1">
         <v>-11</v>
       </c>
-      <c r="E136" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A137" t="s">
+      <c r="E136" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F136" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G136" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A137" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B137" t="s">
-        <v>50</v>
-      </c>
-      <c r="C137">
-        <v>0.16300000000000001</v>
-      </c>
-      <c r="D137">
-        <v>-11</v>
-      </c>
-      <c r="E137" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A138" t="s">
+      <c r="B137" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C137" s="1">
+        <v>0.27400000000000002</v>
+      </c>
+      <c r="D137" s="1">
+        <v>-9</v>
+      </c>
+      <c r="E137" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F137" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G137" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A138" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B138" t="s">
-        <v>55</v>
-      </c>
-      <c r="C138">
-        <v>0.17899999999999999</v>
-      </c>
-      <c r="D138">
-        <v>1</v>
-      </c>
-      <c r="E138" t="s">
-        <v>21</v>
+      <c r="B138" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C138" s="1">
+        <v>0.35</v>
+      </c>
+      <c r="D138" s="1">
+        <v>-10</v>
+      </c>
+      <c r="E138" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F138" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G138" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.2">
@@ -5589,13 +5641,13 @@
         <v>58</v>
       </c>
       <c r="B139" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C139">
-        <v>0.23499999999999999</v>
+        <v>0.13100000000000001</v>
       </c>
       <c r="D139">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E139" t="s">
         <v>21</v>
@@ -5606,39 +5658,33 @@
         <v>58</v>
       </c>
       <c r="B140" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C140">
-        <v>0.21299999999999999</v>
+        <v>0.33800000000000002</v>
       </c>
       <c r="D140">
-        <v>11</v>
+        <v>-11</v>
       </c>
       <c r="E140" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="141" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A141" s="1" t="s">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A141" t="s">
         <v>58</v>
       </c>
-      <c r="B141" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C141" s="1">
-        <v>0.34100000000000003</v>
-      </c>
-      <c r="D141" s="1">
+      <c r="B141" t="s">
+        <v>50</v>
+      </c>
+      <c r="C141">
+        <v>0.16300000000000001</v>
+      </c>
+      <c r="D141">
         <v>-11</v>
       </c>
-      <c r="E141" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F141" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G141" s="1" t="s">
-        <v>6</v>
+      <c r="E141" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.2">
@@ -5646,13 +5692,13 @@
         <v>58</v>
       </c>
       <c r="B142" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="C142">
-        <v>0.20899999999999999</v>
+        <v>0.17899999999999999</v>
       </c>
       <c r="D142">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E142" t="s">
         <v>21</v>
@@ -5663,39 +5709,33 @@
         <v>58</v>
       </c>
       <c r="B143" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C143">
-        <v>0.156</v>
+        <v>0.23499999999999999</v>
       </c>
       <c r="D143">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E143" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="144" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A144" s="1" t="s">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A144" t="s">
         <v>58</v>
       </c>
-      <c r="B144" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C144" s="1">
-        <v>0.70399999999999996</v>
-      </c>
-      <c r="D144" s="1">
-        <v>0</v>
-      </c>
-      <c r="E144" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F144" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G144" s="1" t="s">
-        <v>6</v>
+      <c r="B144" t="s">
+        <v>46</v>
+      </c>
+      <c r="C144">
+        <v>0.21299999999999999</v>
+      </c>
+      <c r="D144">
+        <v>11</v>
+      </c>
+      <c r="E144" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="145" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -5703,13 +5743,13 @@
         <v>58</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C145" s="1">
-        <v>0.48899999999999999</v>
+        <v>0.34100000000000003</v>
       </c>
       <c r="D145" s="1">
-        <v>0</v>
+        <v>-11</v>
       </c>
       <c r="E145" s="1" t="s">
         <v>6</v>
@@ -5721,27 +5761,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="146" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A146" s="1" t="s">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A146" t="s">
         <v>58</v>
       </c>
-      <c r="B146" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C146" s="1">
-        <v>0.73699999999999999</v>
-      </c>
-      <c r="D146" s="1">
-        <v>0</v>
-      </c>
-      <c r="E146" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F146" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G146" s="1" t="s">
-        <v>6</v>
+      <c r="B146" t="s">
+        <v>24</v>
+      </c>
+      <c r="C146">
+        <v>0.20899999999999999</v>
+      </c>
+      <c r="D146">
+        <v>9</v>
+      </c>
+      <c r="E146" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.2">
@@ -5749,13 +5783,13 @@
         <v>58</v>
       </c>
       <c r="B147" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="C147">
-        <v>5.8000000000000003E-2</v>
+        <v>0.156</v>
       </c>
       <c r="D147">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E147" t="s">
         <v>21</v>
@@ -5766,13 +5800,13 @@
         <v>58</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="C148" s="1">
-        <v>0.19600000000000001</v>
+        <v>0.70399999999999996</v>
       </c>
       <c r="D148" s="1">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="E148" s="1" t="s">
         <v>6</v>
@@ -5781,7 +5815,7 @@
         <v>6</v>
       </c>
       <c r="G148" s="1" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
     <row r="149" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -5789,13 +5823,13 @@
         <v>58</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="C149" s="1">
-        <v>0.376</v>
+        <v>0.48899999999999999</v>
       </c>
       <c r="D149" s="1">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="E149" s="1" t="s">
         <v>6</v>
@@ -5807,37 +5841,43 @@
         <v>6</v>
       </c>
     </row>
-    <row r="150" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A150" s="2" t="s">
+    <row r="150" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A150" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B150" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C150" s="2">
+      <c r="B150" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C150" s="1">
+        <v>0.73699999999999999</v>
+      </c>
+      <c r="D150" s="1">
         <v>0</v>
       </c>
-      <c r="D150" s="2">
-        <v>0</v>
-      </c>
-      <c r="E150" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="151" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A151" s="2" t="s">
+      <c r="E150" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F150" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G150" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A151" t="s">
         <v>58</v>
       </c>
-      <c r="B151" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C151" s="2">
-        <v>0.253</v>
-      </c>
-      <c r="D151" s="2">
-        <v>5</v>
-      </c>
-      <c r="E151" s="2" t="s">
+      <c r="B151" t="s">
+        <v>69</v>
+      </c>
+      <c r="C151">
+        <v>5.8000000000000003E-2</v>
+      </c>
+      <c r="D151">
+        <v>4</v>
+      </c>
+      <c r="E151" t="s">
         <v>21</v>
       </c>
     </row>
@@ -5846,13 +5886,13 @@
         <v>58</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="C152" s="1">
-        <v>0.188</v>
+        <v>0.19600000000000001</v>
       </c>
       <c r="D152" s="1">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="E152" s="1" t="s">
         <v>6</v>
@@ -5864,44 +5904,44 @@
         <v>21</v>
       </c>
     </row>
-    <row r="153" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A153" s="2" t="s">
+    <row r="153" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A153" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B153" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C153" s="2">
-        <v>0.14599999999999999</v>
-      </c>
-      <c r="D153" s="2">
-        <v>11</v>
-      </c>
-      <c r="E153" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="154" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A154" s="1" t="s">
+      <c r="B153" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C153" s="1">
+        <v>0.376</v>
+      </c>
+      <c r="D153" s="1">
+        <v>-5</v>
+      </c>
+      <c r="E153" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F153" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G153" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A154" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B154" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C154" s="1">
-        <v>0.20599999999999999</v>
-      </c>
-      <c r="D154" s="1">
-        <v>-2</v>
-      </c>
-      <c r="E154" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F154" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G154" s="1" t="s">
-        <v>6</v>
+      <c r="B154" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C154" s="2">
+        <v>0</v>
+      </c>
+      <c r="D154" s="2">
+        <v>0</v>
+      </c>
+      <c r="E154" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="155" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -5909,32 +5949,38 @@
         <v>58</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C155" s="2">
-        <v>0.14899999999999999</v>
+        <v>0.253</v>
       </c>
       <c r="D155" s="2">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E155" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="156" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A156" s="2" t="s">
+    <row r="156" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A156" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B156" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C156" s="2">
-        <v>0.112</v>
-      </c>
-      <c r="D156" s="2">
-        <v>-3</v>
-      </c>
-      <c r="E156" s="2" t="s">
+      <c r="B156" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C156" s="1">
+        <v>0.188</v>
+      </c>
+      <c r="D156" s="1">
+        <v>-2</v>
+      </c>
+      <c r="E156" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F156" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G156" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -5943,13 +5989,13 @@
         <v>58</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C157" s="2">
-        <v>0.129</v>
+        <v>0.14599999999999999</v>
       </c>
       <c r="D157" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E157" s="2" t="s">
         <v>21</v>
@@ -5960,13 +6006,13 @@
         <v>58</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C158" s="1">
-        <v>0.35199999999999998</v>
+        <v>0.20599999999999999</v>
       </c>
       <c r="D158" s="1">
-        <v>-7</v>
+        <v>-2</v>
       </c>
       <c r="E158" s="1" t="s">
         <v>6</v>
@@ -5978,21 +6024,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="159" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A159" s="1" t="s">
+    <row r="159" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A159" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B159" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C159" s="1">
-        <v>0.54600000000000004</v>
-      </c>
-      <c r="D159" s="1">
-        <v>-5</v>
-      </c>
-      <c r="E159" s="1" t="s">
-        <v>6</v>
+      <c r="B159" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C159" s="2">
+        <v>0.14899999999999999</v>
+      </c>
+      <c r="D159" s="2">
+        <v>12</v>
+      </c>
+      <c r="E159" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="160" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -6000,13 +6046,13 @@
         <v>58</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="C160" s="2">
-        <v>0.184</v>
+        <v>0.112</v>
       </c>
       <c r="D160" s="2">
-        <v>-7</v>
+        <v>-3</v>
       </c>
       <c r="E160" s="2" t="s">
         <v>21</v>
@@ -6017,10 +6063,10 @@
         <v>58</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="C161" s="2">
-        <v>0.13900000000000001</v>
+        <v>0.129</v>
       </c>
       <c r="D161" s="2">
         <v>12</v>
@@ -6034,13 +6080,13 @@
         <v>58</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C162" s="1">
-        <v>0.33300000000000002</v>
+        <v>0.35199999999999998</v>
       </c>
       <c r="D162" s="1">
-        <v>-2</v>
+        <v>-7</v>
       </c>
       <c r="E162" s="1" t="s">
         <v>6</v>
@@ -6052,44 +6098,38 @@
         <v>6</v>
       </c>
     </row>
-    <row r="163" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A163" s="2" t="s">
+    <row r="163" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A163" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B163" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C163" s="2">
-        <v>0.191</v>
-      </c>
-      <c r="D163" s="2">
-        <v>3</v>
-      </c>
-      <c r="E163" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="164" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A164" s="1" t="s">
+      <c r="B163" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C163" s="1">
+        <v>0.54600000000000004</v>
+      </c>
+      <c r="D163" s="1">
+        <v>-5</v>
+      </c>
+      <c r="E163" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A164" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B164" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C164" s="1">
-        <v>0.219</v>
-      </c>
-      <c r="D164" s="1">
-        <v>-5</v>
-      </c>
-      <c r="E164" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F164" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G164" s="1" t="s">
-        <v>6</v>
+      <c r="B164" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C164" s="2">
+        <v>0.184</v>
+      </c>
+      <c r="D164" s="2">
+        <v>-7</v>
+      </c>
+      <c r="E164" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="165" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -6097,10 +6137,10 @@
         <v>58</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C165" s="2">
-        <v>0.17199999999999999</v>
+        <v>0.13900000000000001</v>
       </c>
       <c r="D165" s="2">
         <v>12</v>
@@ -6114,10 +6154,10 @@
         <v>58</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C166" s="1">
-        <v>0.22</v>
+        <v>0.33300000000000002</v>
       </c>
       <c r="D166" s="1">
         <v>-2</v>
@@ -6132,38 +6172,164 @@
         <v>6</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A167" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B167" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C167" s="2">
+        <v>0.191</v>
+      </c>
+      <c r="D167" s="2">
+        <v>3</v>
+      </c>
+      <c r="E167" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A168" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B168" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C168" s="1">
+        <v>0.219</v>
+      </c>
+      <c r="D168" s="1">
+        <v>-5</v>
+      </c>
+      <c r="E168" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F168" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G168" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A169" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B169" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C169" s="2">
+        <v>0.17199999999999999</v>
+      </c>
+      <c r="D169" s="2">
+        <v>12</v>
+      </c>
+      <c r="E169" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A170" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B170" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C170" s="1">
+        <v>0.22</v>
+      </c>
+      <c r="D170" s="1">
+        <v>-2</v>
+      </c>
+      <c r="E170" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F170" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G170" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A171" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B171" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C167" s="2">
+      <c r="C171" s="2">
         <v>0.2</v>
       </c>
-      <c r="D167" s="2">
+      <c r="D171" s="2">
         <v>12</v>
       </c>
-      <c r="E167" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="168" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A168" s="2" t="s">
+      <c r="E171" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A172" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B168" s="2" t="s">
+      <c r="B172" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C168" s="2">
+      <c r="C172" s="2">
         <v>0.155</v>
       </c>
-      <c r="D168" s="2">
+      <c r="D172" s="2">
         <v>-5</v>
       </c>
-      <c r="E168" s="2" t="s">
-        <v>21</v>
+      <c r="E172" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A173" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B173" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C173" s="1">
+        <v>0.46800000000000003</v>
+      </c>
+      <c r="D173" s="1">
+        <v>-6</v>
+      </c>
+      <c r="E173" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F173" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G173" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A174" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B174" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C174" s="1">
+        <v>0.53600000000000003</v>
+      </c>
+      <c r="D174" s="1">
+        <v>-6</v>
+      </c>
+      <c r="E174" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F174" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G174" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
forgot the parameters excel last commit
</commit_message>
<xml_diff>
--- a/parameters_CCM.xlsx
+++ b/parameters_CCM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rodemann/Algal_EDM/Algal_blooms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E677FB-D1CF-5445-A9BB-28B136E503EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{208AE150-6A64-7842-90E5-B5CA4376350D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="6" xr2:uid="{96C955FB-9A51-4D0B-AF49-129559A448B6}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="7" xr2:uid="{96C955FB-9A51-4D0B-AF49-129559A448B6}"/>
   </bookViews>
   <sheets>
     <sheet name="Run1" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Run4" sheetId="5" r:id="rId5"/>
     <sheet name="Surrogate_results" sheetId="6" r:id="rId6"/>
     <sheet name="leadlag_results" sheetId="7" r:id="rId7"/>
+    <sheet name="Final_results" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="936" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1191" uniqueCount="167">
   <si>
     <t>Variable</t>
   </si>
@@ -338,6 +339,210 @@
   </si>
   <si>
     <t>dcbre</t>
+  </si>
+  <si>
+    <t>Graph</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Hypothesis</t>
+  </si>
+  <si>
+    <t>Use?</t>
+  </si>
+  <si>
+    <t>max_lag</t>
+  </si>
+  <si>
+    <t>EDM at max lag?</t>
+  </si>
+  <si>
+    <t>number</t>
+  </si>
+  <si>
+    <t>1a</t>
+  </si>
+  <si>
+    <t>marsh</t>
+  </si>
+  <si>
+    <t>coastal lakes</t>
+  </si>
+  <si>
+    <t>1b</t>
+  </si>
+  <si>
+    <t>1c</t>
+  </si>
+  <si>
+    <t>gulf of mexico</t>
+  </si>
+  <si>
+    <t>1d</t>
+  </si>
+  <si>
+    <t>florida bay itself</t>
+  </si>
+  <si>
+    <t>mangrove rim</t>
+  </si>
+  <si>
+    <t>2a</t>
+  </si>
+  <si>
+    <t>acdocarea</t>
+  </si>
+  <si>
+    <t>acdocnorthing</t>
+  </si>
+  <si>
+    <t>actnnorthing</t>
+  </si>
+  <si>
+    <t>amaxstagearea</t>
+  </si>
+  <si>
+    <t>cchlarea</t>
+  </si>
+  <si>
+    <t>proving method works</t>
+  </si>
+  <si>
+    <t>pmw</t>
+  </si>
+  <si>
+    <t>areadcbre</t>
+  </si>
+  <si>
+    <t>areaetoc</t>
+  </si>
+  <si>
+    <t>areagchl</t>
+  </si>
+  <si>
+    <t>arearchl</t>
+  </si>
+  <si>
+    <t>gchlrchl</t>
+  </si>
+  <si>
+    <t>1b, 1c</t>
+  </si>
+  <si>
+    <t>gpHgchl</t>
+  </si>
+  <si>
+    <t>1b?</t>
+  </si>
+  <si>
+    <t>gsalgchl</t>
+  </si>
+  <si>
+    <t>gsalrchl</t>
+  </si>
+  <si>
+    <t>gsmeanstagearea</t>
+  </si>
+  <si>
+    <t>gtngchl</t>
+  </si>
+  <si>
+    <t>gtn</t>
+  </si>
+  <si>
+    <t>gtnrchl</t>
+  </si>
+  <si>
+    <t>gtocarea</t>
+  </si>
+  <si>
+    <t>gtoc</t>
+  </si>
+  <si>
+    <t>gtocgchl</t>
+  </si>
+  <si>
+    <t>gtocrchl</t>
+  </si>
+  <si>
+    <t>gtpgchl</t>
+  </si>
+  <si>
+    <t>gtp</t>
+  </si>
+  <si>
+    <t>gtprchl</t>
+  </si>
+  <si>
+    <t>mcdocarea</t>
+  </si>
+  <si>
+    <t>mmaxstagearea</t>
+  </si>
+  <si>
+    <t>rchlarea</t>
+  </si>
+  <si>
+    <t>cchlrchl</t>
+  </si>
+  <si>
+    <t>cnh4rchl</t>
+  </si>
+  <si>
+    <t>cturbrchl</t>
+  </si>
+  <si>
+    <t>dcbrerchl</t>
+  </si>
+  <si>
+    <t>rchletn</t>
+  </si>
+  <si>
+    <t>etn</t>
+  </si>
+  <si>
+    <t>rchletp</t>
+  </si>
+  <si>
+    <t>etp</t>
+  </si>
+  <si>
+    <t>rchleturb</t>
+  </si>
+  <si>
+    <t>rsalgchl</t>
+  </si>
+  <si>
+    <t>rsalnorthing</t>
+  </si>
+  <si>
+    <t>rtnarea</t>
+  </si>
+  <si>
+    <t>rtn</t>
+  </si>
+  <si>
+    <t>rtnrchl</t>
+  </si>
+  <si>
+    <t>rtoc</t>
+  </si>
+  <si>
+    <t>rtocarea</t>
+  </si>
+  <si>
+    <t>rtocrchl</t>
+  </si>
+  <si>
+    <t>rtparea</t>
+  </si>
+  <si>
+    <t>rtp</t>
+  </si>
+  <si>
+    <t>rtprchl</t>
   </si>
 </sst>
 </file>
@@ -6335,4 +6540,989 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{559CCFFA-51A4-2641-843E-EE14BED60336}">
+  <dimension ref="A1:L40"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" customWidth="1"/>
+    <col min="3" max="4" width="13.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.1640625" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="18.5" customWidth="1"/>
+    <col min="11" max="11" width="30" customWidth="1"/>
+    <col min="12" max="12" width="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F1" t="s">
+        <v>102</v>
+      </c>
+      <c r="G1" t="s">
+        <v>104</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="1">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>122</v>
+      </c>
+      <c r="F4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" s="1">
+        <v>10</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6" t="s">
+        <v>122</v>
+      </c>
+      <c r="F6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7">
+        <v>4</v>
+      </c>
+      <c r="E7" t="s">
+        <v>122</v>
+      </c>
+      <c r="F7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8">
+        <v>6</v>
+      </c>
+      <c r="E8" t="s">
+        <v>122</v>
+      </c>
+      <c r="F8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>133</v>
+      </c>
+      <c r="B9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>109</v>
+      </c>
+      <c r="F9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>137</v>
+      </c>
+      <c r="B10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D10">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>128</v>
+      </c>
+      <c r="F10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>144</v>
+      </c>
+      <c r="B11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11" t="s">
+        <v>109</v>
+      </c>
+      <c r="F11" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>145</v>
+      </c>
+      <c r="B12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>109</v>
+      </c>
+      <c r="F12" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" s="1">
+        <v>4</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>162</v>
+      </c>
+      <c r="B15" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" t="s">
+        <v>161</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15" t="s">
+        <v>122</v>
+      </c>
+      <c r="F15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D16" s="1">
+        <v>0</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" s="1">
+        <v>4</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>131</v>
+      </c>
+      <c r="B18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>130</v>
+      </c>
+      <c r="F18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>134</v>
+      </c>
+      <c r="B19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" t="s">
+        <v>135</v>
+      </c>
+      <c r="D19">
+        <v>8</v>
+      </c>
+      <c r="E19" t="s">
+        <v>122</v>
+      </c>
+      <c r="F19" t="s">
+        <v>21</v>
+      </c>
+      <c r="G19" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>139</v>
+      </c>
+      <c r="B20" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>138</v>
+      </c>
+      <c r="D20">
+        <v>7</v>
+      </c>
+      <c r="E20" t="s">
+        <v>122</v>
+      </c>
+      <c r="F20" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="D21" s="1">
+        <v>10</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>156</v>
+      </c>
+      <c r="B22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>57</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22" t="s">
+        <v>115</v>
+      </c>
+      <c r="F22" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="1">
+        <v>7</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>118</v>
+      </c>
+      <c r="B24" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24">
+        <v>7</v>
+      </c>
+      <c r="E24" t="s">
+        <v>109</v>
+      </c>
+      <c r="F24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>157</v>
+      </c>
+      <c r="B25" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25">
+        <v>3</v>
+      </c>
+      <c r="E25" t="s">
+        <v>115</v>
+      </c>
+      <c r="F25" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D26" s="1">
+        <v>11</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>132</v>
+      </c>
+      <c r="B27" t="s">
+        <v>58</v>
+      </c>
+      <c r="C27" t="s">
+        <v>18</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27" t="s">
+        <v>130</v>
+      </c>
+      <c r="F27" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>136</v>
+      </c>
+      <c r="B28" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" t="s">
+        <v>135</v>
+      </c>
+      <c r="D28">
+        <v>9</v>
+      </c>
+      <c r="E28" t="s">
+        <v>128</v>
+      </c>
+      <c r="F28" t="s">
+        <v>21</v>
+      </c>
+      <c r="G28" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>140</v>
+      </c>
+      <c r="B29" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" t="s">
+        <v>138</v>
+      </c>
+      <c r="D29">
+        <v>9</v>
+      </c>
+      <c r="E29" t="s">
+        <v>128</v>
+      </c>
+      <c r="F29" t="s">
+        <v>21</v>
+      </c>
+      <c r="G29" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="D30" s="1">
+        <v>10</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>147</v>
+      </c>
+      <c r="B31" t="s">
+        <v>58</v>
+      </c>
+      <c r="C31" t="s">
+        <v>84</v>
+      </c>
+      <c r="D31">
+        <v>6</v>
+      </c>
+      <c r="E31" t="s">
+        <v>112</v>
+      </c>
+      <c r="F31" t="s">
+        <v>21</v>
+      </c>
+      <c r="G31" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D32" s="1">
+        <v>5</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>149</v>
+      </c>
+      <c r="B33" t="s">
+        <v>58</v>
+      </c>
+      <c r="C33" t="s">
+        <v>80</v>
+      </c>
+      <c r="D33">
+        <v>2</v>
+      </c>
+      <c r="E33" t="s">
+        <v>112</v>
+      </c>
+      <c r="F33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G33" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D34" s="1">
+        <v>6</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>151</v>
+      </c>
+      <c r="B35" t="s">
+        <v>58</v>
+      </c>
+      <c r="C35" t="s">
+        <v>152</v>
+      </c>
+      <c r="D35">
+        <v>2</v>
+      </c>
+      <c r="E35" t="s">
+        <v>112</v>
+      </c>
+      <c r="F35" t="s">
+        <v>21</v>
+      </c>
+      <c r="G35" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D36" s="1">
+        <v>2</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>155</v>
+      </c>
+      <c r="B37" t="s">
+        <v>58</v>
+      </c>
+      <c r="C37" t="s">
+        <v>92</v>
+      </c>
+      <c r="D37">
+        <v>5</v>
+      </c>
+      <c r="E37" t="s">
+        <v>112</v>
+      </c>
+      <c r="F37" t="s">
+        <v>21</v>
+      </c>
+      <c r="G37" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D38" s="1">
+        <v>0</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>163</v>
+      </c>
+      <c r="B39" t="s">
+        <v>58</v>
+      </c>
+      <c r="C39" t="s">
+        <v>161</v>
+      </c>
+      <c r="D39">
+        <v>0</v>
+      </c>
+      <c r="E39" t="s">
+        <v>122</v>
+      </c>
+      <c r="F39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G39" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D40" s="1">
+        <v>0</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G40">
+    <sortCondition ref="B1:B40"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated with Johnson data, testing Garfield pH
</commit_message>
<xml_diff>
--- a/parameters_CCM.xlsx
+++ b/parameters_CCM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rodemann/Algal_EDM/Algal_blooms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{208AE150-6A64-7842-90E5-B5CA4376350D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9938E355-70FA-CD42-91D6-9A782AB7797D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="7" xr2:uid="{96C955FB-9A51-4D0B-AF49-129559A448B6}"/>
   </bookViews>
@@ -6635,7 +6635,7 @@
         <v>6</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>108</v>
@@ -6644,32 +6644,32 @@
         <v>109</v>
       </c>
     </row>
-    <row r="4" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="4" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B4" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="1">
         <v>1</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="F4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G4" t="s">
-        <v>21</v>
-      </c>
-      <c r="K4" s="2" t="s">
+      <c r="F4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="1" t="s">
         <v>110</v>
       </c>
     </row>

</xml_diff>